<commit_message>
auto: sync reports 2026-05-05 15:54
</commit_message>
<xml_diff>
--- a/feedback-reports/Java_Development_Certificate_Program.xlsx
+++ b/feedback-reports/Java_Development_Certificate_Program.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Website-Feedback\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Feedback-App\feedback-reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="14_{993EE370-A134-4F5E-8879-CE421C0D6BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F413FD7-906B-4FC2-86F8-001E16EA7801}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="14_{993EE370-A134-4F5E-8879-CE421C0D6BDF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECC2CFA6-A266-4746-A977-B14CC299631D}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="117">
   <si>
     <t>Program Name:</t>
   </si>
@@ -223,6 +223,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">1.Core Java Foundations
@@ -233,6 +234,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Build programs using Core Java with decision making, loops, arrays, strings, recursion, and basic searching and sorting to solve real problems.
@@ -244,6 +246,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">2.Object-Oriented Programming
@@ -254,6 +257,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Design applications using object-oriented concepts and exception handling to create structured, real-world solutions.</t>
@@ -347,6 +351,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Replace with
 </t>
@@ -357,6 +362,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">• Unit Testing and Collections
 </t>
@@ -366,6 +372,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Write unit tests, enforce type safety with generics, and organize data using Java Collections with sorting.
 </t>
@@ -376,6 +383,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">• Functional Programming and Data Processing
 </t>
@@ -385,6 +393,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Apply lambdas and functional interfaces, and process data using Streams with null-safe handling.</t>
     </r>
@@ -486,12 +495,15 @@
   <si>
     <t>Add a closing outcome bullet: 'Be job-ready for the entry-level Java Developer role by combining technical skills with professional best practices and the right engineering mindset.'</t>
   </si>
+  <si>
+    <t>Status</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,22 +516,26 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -535,6 +551,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -556,19 +573,29 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -591,6 +618,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAEEF3"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -633,7 +666,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -671,6 +704,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -975,20 +1014,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:I33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="7" width="43.28515625" customWidth="1"/>
+    <col min="7" max="7" width="43.33203125" customWidth="1"/>
     <col min="8" max="8" width="71" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="33.75" customHeight="1">
+    <row r="1" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1004,11 +1043,11 @@
       </c>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="6"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:9" ht="33.75" customHeight="1">
+    <row r="2" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1019,11 +1058,11 @@
       <c r="D2" s="5"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="6"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
       <c r="I2" s="6"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1043,10 +1082,13 @@
         <v>10</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="H3" s="15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="86.25">
+    <row r="4" spans="1:9" ht="69" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1</v>
       </c>
@@ -1064,7 +1106,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="82.9">
+    <row r="5" spans="1:9" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>2</v>
       </c>
@@ -1084,7 +1126,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="187.5">
+    <row r="6" spans="1:9" ht="179.4" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>3</v>
       </c>
@@ -1102,7 +1144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>4</v>
       </c>
@@ -1122,7 +1164,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>5</v>
       </c>
@@ -1140,7 +1182,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="28.5">
+    <row r="9" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>6</v>
       </c>
@@ -1158,7 +1200,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="28.5">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>7</v>
       </c>
@@ -1176,7 +1218,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="57.75">
+    <row r="11" spans="1:9" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>8</v>
       </c>
@@ -1196,7 +1238,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="213">
+    <row r="12" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>9</v>
       </c>
@@ -1214,7 +1256,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="28.5">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>10</v>
       </c>
@@ -1232,7 +1274,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="48">
+    <row r="14" spans="1:9" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>11</v>
       </c>
@@ -1252,7 +1294,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="115.5">
+    <row r="15" spans="1:9" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>12</v>
       </c>
@@ -1272,7 +1314,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="137.25">
+    <row r="16" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>13</v>
       </c>
@@ -1290,7 +1332,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="28.5">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>14</v>
       </c>
@@ -1308,7 +1350,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="96">
+    <row r="18" spans="1:7" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>15</v>
       </c>
@@ -1328,7 +1370,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="101.25">
+    <row r="19" spans="1:7" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>16</v>
       </c>
@@ -1349,7 +1391,7 @@
       </c>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:7" ht="152.25">
+    <row r="20" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>17</v>
       </c>
@@ -1367,7 +1409,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="28.5">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>18</v>
       </c>
@@ -1385,7 +1427,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="60">
+    <row r="22" spans="1:7" ht="66" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>19</v>
       </c>
@@ -1405,7 +1447,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="28.5">
+    <row r="23" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>20</v>
       </c>
@@ -1423,7 +1465,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="101.25">
+    <row r="24" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>21</v>
       </c>
@@ -1443,7 +1485,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="173.25">
+    <row r="25" spans="1:7" ht="165.6" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
         <v>22</v>
       </c>
@@ -1461,7 +1503,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="28.5">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>23</v>
       </c>
@@ -1479,7 +1521,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="96">
+    <row r="27" spans="1:7" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>24</v>
       </c>
@@ -1499,7 +1541,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="57.75">
+    <row r="28" spans="1:7" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
         <v>25</v>
       </c>
@@ -1517,7 +1559,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="72">
+    <row r="29" spans="1:7" ht="69" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
         <v>26</v>
       </c>
@@ -1537,7 +1579,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="86.25">
+    <row r="30" spans="1:7" ht="69" x14ac:dyDescent="0.3">
       <c r="A30" s="8">
         <v>27</v>
       </c>
@@ -1557,7 +1599,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="351">
+    <row r="31" spans="1:7" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
         <v>28</v>
       </c>
@@ -1577,7 +1619,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="72">
+    <row r="32" spans="1:7" ht="69" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
         <v>29</v>
       </c>
@@ -1597,7 +1639,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="144">
+    <row r="33" spans="1:8" ht="138" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>30</v>
       </c>
@@ -1616,8 +1658,6 @@
       </c>
       <c r="H33" s="3"/>
     </row>
-    <row r="34" spans="1:8" ht="15"/>
-    <row r="35" spans="1:8" ht="15"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{3D5E3770-7B3A-46CB-8344-5C60E164B9D6}"/>
@@ -1633,15 +1673,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008081BF50E816F94B87E854E2907183B0" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f6f57204d0cc9b1c65f7ab94eaa7dcc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8b8ad293-1655-4b1e-95cd-578b981aff66" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ed196dee19b1527225c6137bc92e865" ns2:_="">
     <xsd:import namespace="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
@@ -1803,14 +1834,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCB0A042-CF97-49A2-B019-0CFB7043FEE1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCB0A042-CF97-49A2-B019-0CFB7043FEE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354ECB66-1915-4F9E-BB56-038B20F3916E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97220449-414E-44C9-BC04-9A4AAE96FA91}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97220449-414E-44C9-BC04-9A4AAE96FA91}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354ECB66-1915-4F9E-BB56-038B20F3916E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>